<commit_message>
Site updated: 2021-09-28 16:42:29
</commit_message>
<xml_diff>
--- a/games/life/data/specialthanks-afd.xlsx
+++ b/games/life/data/specialthanks-afd.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\84694\Desktop\人生重来\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269F04D8-F596-496A-BF00-B8BE09FA7437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{432123CF-23A5-4A7E-BD8A-CE4E8D292F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="606">
   <si>
     <t>group</t>
   </si>
@@ -2159,6 +2159,69 @@
   </si>
   <si>
     <t>#ffccff</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>coz</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>迪拜小泥人</t>
+  </si>
+  <si>
+    <t>各自安好</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多多支持国产游戏加油</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DialEctic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>请让小翼在学会儿</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>鱼饼</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Golz</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>不吃香菜不订断更</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kxu3nive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>罡风甚是喧嚣</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Liangbi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>debuff</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>方飞</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>雪莉丨星凌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>披坚执锐</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2499,7 +2562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D545"/>
+  <dimension ref="A1:D560"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.88671875" style="1" customWidth="1"/>
@@ -6999,12 +7062,135 @@
         <v>587</v>
       </c>
     </row>
-    <row r="545" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="545" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A545" s="1">
         <v>2</v>
       </c>
       <c r="B545" s="3" t="s">
         <v>588</v>
+      </c>
+    </row>
+    <row r="546" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A546" s="1">
+        <v>2</v>
+      </c>
+      <c r="B546" s="3" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="547" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A547" s="1">
+        <v>2</v>
+      </c>
+      <c r="B547" s="3" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="548" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A548" s="1">
+        <v>1</v>
+      </c>
+      <c r="B548" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="C548" s="3" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="549" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A549" s="1">
+        <v>2</v>
+      </c>
+      <c r="B549" s="3" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="550" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A550" s="1">
+        <v>2</v>
+      </c>
+      <c r="B550" s="3" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="551" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A551" s="1">
+        <v>2</v>
+      </c>
+      <c r="B551" s="3" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="552" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A552" s="1">
+        <v>2</v>
+      </c>
+      <c r="B552" s="3" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="553" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A553" s="1">
+        <v>2</v>
+      </c>
+      <c r="B553" s="3" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="554" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A554" s="1">
+        <v>2</v>
+      </c>
+      <c r="B554" s="3" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="555" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A555" s="1">
+        <v>2</v>
+      </c>
+      <c r="B555" s="3" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="556" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A556" s="1">
+        <v>2</v>
+      </c>
+      <c r="B556" s="3" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="557" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A557" s="1">
+        <v>2</v>
+      </c>
+      <c r="B557" s="3" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="558" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A558" s="1">
+        <v>2</v>
+      </c>
+      <c r="B558" s="3" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="559" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A559" s="1">
+        <v>2</v>
+      </c>
+      <c r="B559" s="3" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="560" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A560" s="1">
+        <v>2</v>
+      </c>
+      <c r="B560" s="3" t="s">
+        <v>605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>